<commit_message>
edim-ai-blueprint: 메뉴정의서 2차 검증 — Purchasing/Material Head Tab 분리, 표시 경로 비고 보강
- 2차 전수 대조: breadcrumb 8경로·ERP Head Tab 10종·프로세스 코드 41종 모두 커버 확인
- Purchasing·Material 병합 오류 수정 (원문은 별도 Head Tab)
- M-4-1 실제 표시 경로(Drawing Info. > Production Design Management) 및 M-4-2 하위 실체 비고
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_메뉴정의서.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_메뉴정의서.xlsx
@@ -2076,7 +2076,7 @@
       </c>
       <c r="K27" s="7" t="inlineStr">
         <is>
-          <t>Drawing Editor</t>
+          <t>Drawing Editor — 표시 경로: Drawing Info. &gt; Production Design Management &gt; Design &gt; Check &gt; Approve &gt; Accepted</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,11 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="K28" s="7" t="inlineStr"/>
+      <c r="K28" s="7" t="inlineStr">
+        <is>
+          <t>하위 실체: Design·Manufacturing·Material·Quality (제품별 Work Process Tree)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n">
@@ -3081,7 +3085,7 @@
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Purchasing·Material</t>
+          <t>Purchasing</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
@@ -3132,7 +3136,7 @@
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Purchasing·Material</t>
+          <t>Purchasing</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
@@ -3183,7 +3187,7 @@
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Purchasing·Material</t>
+          <t>Material</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
@@ -3234,7 +3238,7 @@
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Purchasing·Material</t>
+          <t>Material</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
@@ -3285,7 +3289,7 @@
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Purchasing·Material</t>
+          <t>Material</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
@@ -3336,7 +3340,7 @@
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Purchasing·Material</t>
+          <t>Purchasing</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">

</xml_diff>

<commit_message>
edim-ai-blueprint: 메뉴 3차 검증 (+7 → 97) + 와이어프레임 6화면 추가 (W-11~W-16)
- 신규 누락: ERP Process/DB/Form Set-up(슬라이드17 5-1~5-3), 단가 관리(74/75),
  Toolbox 검색·AI질의(27노트), History 조회(57/72), 보안 설정(58)
- 화면설계서 v0.2: Document Mgmt, 승인함, 단가 관리, ERP Process Set-up,
  건축 설비 Duct 자동배치, Mobile App(3폰 프레임) — 16화면
- 메뉴↔화면 ID 재배정 (M-5-4→W-11, M-15-2→W-12, M-12-5→W-13 등)
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_메뉴정의서.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_메뉴정의서.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="메뉴목록" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'메뉴목록'!$A$1:$K$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'메뉴목록'!$A$1:$K$98</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -598,7 +598,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>90개</t>
+          <t>97개</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K91"/>
+  <dimension ref="A1:K98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1407,22 +1407,22 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>M-2-1</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>CPQ Set-up</t>
+          <t>M-1-8</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>EDIM Toolbox</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>CPQ</t>
+          <t>지원 도구</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Selection</t>
+          <t>인터넷 검색·AI 질의응답</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -1432,25 +1432,29 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>S-3-1</t>
+          <t>S-2-2</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>CPQ-011</t>
+          <t>TBX-015, AI-007</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>SETUP</t>
+          <t>전체</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="K15" s="7" t="inlineStr"/>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>슬라이드 27 발표자 노트 — 내부 자료 검색·응답용</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
@@ -1458,7 +1462,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>M-2-2</t>
+          <t>M-2-1</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -1473,7 +1477,7 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Technical</t>
+          <t>Selection</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -1483,12 +1487,12 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>S-3-2</t>
+          <t>S-3-1</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>CPQ-012</t>
+          <t>CPQ-011</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -1509,7 +1513,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>M-2-3</t>
+          <t>M-2-2</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -1524,7 +1528,7 @@
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Document</t>
+          <t>Technical</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -1534,7 +1538,7 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>S-3-3</t>
+          <t>S-3-2</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -1560,7 +1564,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>M-2-4</t>
+          <t>M-2-3</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -1575,7 +1579,7 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>Print Set-up</t>
+          <t>Document</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1585,12 +1589,12 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>S-3-4</t>
+          <t>S-3-3</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>CPQ-013</t>
+          <t>CPQ-012</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -1611,7 +1615,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>M-2-5</t>
+          <t>M-2-4</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -1621,12 +1625,12 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>User Management</t>
+          <t>CPQ</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>User Customizing ERP</t>
+          <t>Print Set-up</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -1636,12 +1640,12 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>S-3-5</t>
+          <t>S-3-4</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>ERP-001/016</t>
+          <t>CPQ-013</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -1651,7 +1655,7 @@
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="K19" s="7" t="inlineStr"/>
@@ -1662,37 +1666,37 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>M-3-1</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>Code(TLM) Set-up</t>
+          <t>M-2-5</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>CPQ Set-up</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>User Management</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>Sub Code Spec.</t>
+          <t>User Customizing ERP</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>W-04</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>S-1-1</t>
+          <t>S-3-5</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>CODE-001~004/015</t>
+          <t>ERP-001/016</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
@@ -1702,7 +1706,7 @@
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="K20" s="7" t="inlineStr"/>
@@ -1713,7 +1717,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>M-3-2</t>
+          <t>M-3-1</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
@@ -1728,7 +1732,7 @@
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Sub Code Raw Material·GPI</t>
+          <t>Sub Code Spec.</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -1738,12 +1742,12 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>S-1-2</t>
+          <t>S-1-1</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>CODE-005</t>
+          <t>CODE-001~004/015</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
@@ -1756,11 +1760,7 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="K21" s="7" t="inlineStr">
-        <is>
-          <t>슬라이드 34 breadcrumb: Raw material Or GPI</t>
-        </is>
-      </c>
+      <c r="K21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>M-3-3</t>
+          <t>M-3-2</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Product Code</t>
+          <t>Sub Code Raw Material·GPI</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -1793,12 +1793,12 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>S-1-3</t>
+          <t>S-1-2</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>CODE-006/007</t>
+          <t>CODE-005</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
@@ -1811,7 +1811,11 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="K22" s="7" t="inlineStr"/>
+      <c r="K22" s="7" t="inlineStr">
+        <is>
+          <t>슬라이드 34 breadcrumb: Raw material Or GPI</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
@@ -1819,7 +1823,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>M-3-4</t>
+          <t>M-3-3</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
@@ -1834,22 +1838,22 @@
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Code Relationship</t>
+          <t>Product Code</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>W-05</t>
+          <t>W-04</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>S-1-4</t>
+          <t>S-1-3</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>CODE-008~010</t>
+          <t>CODE-006/007</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
@@ -1862,11 +1866,7 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="K23" s="7" t="inlineStr">
-        <is>
-          <t>관계형 BOM</t>
-        </is>
-      </c>
+      <c r="K23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>M-3-5</t>
+          <t>M-3-4</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
@@ -1889,22 +1889,22 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Arrangement Code</t>
+          <t>Code Relationship</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>W-04</t>
+          <t>W-05</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>S-1-5</t>
+          <t>S-1-4</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>CODE-011</t>
+          <t>CODE-008~010</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -1914,10 +1914,14 @@
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="K24" s="7" t="inlineStr"/>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K24" s="7" t="inlineStr">
+        <is>
+          <t>관계형 BOM</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n">
@@ -1925,7 +1929,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>M-3-6</t>
+          <t>M-3-5</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
@@ -1940,22 +1944,22 @@
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>Arrangement Set-up</t>
+          <t>Arrangement Code</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>W-06</t>
+          <t>W-04</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>S-1-6</t>
+          <t>S-1-5</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>CODE-012</t>
+          <t>CODE-011</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -1976,7 +1980,7 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>M-3-7</t>
+          <t>M-3-6</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
@@ -1986,27 +1990,27 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Table·Variant·Constant·단위계(Metric)</t>
+          <t>Arrangement Set-up</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-06</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>E-4</t>
+          <t>S-1-6</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>TBL-001~006</t>
+          <t>CODE-012</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
@@ -2016,14 +2020,10 @@
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="K26" s="7" t="inlineStr">
-        <is>
-          <t>슬라이드 46 — Constant List·Metric System은 기능정의서 v0.3 보강 필요</t>
-        </is>
-      </c>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K26" s="7" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
@@ -2031,37 +2031,37 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>M-4-1</t>
-        </is>
-      </c>
-      <c r="C27" s="11" t="inlineStr">
-        <is>
-          <t>PLM Set-up</t>
+          <t>M-3-7</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Code(TLM) Set-up</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Design (DWG)</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Table·Variant·Constant·단위계(Metric)</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>W-06</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>S-4-1-1</t>
+          <t>E-4</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>DWG-001~016/022~027</t>
+          <t>TBL-001~006</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
@@ -2071,12 +2071,12 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
         <is>
-          <t>Drawing Editor — 표시 경로: Drawing Info. &gt; Production Design Management &gt; Design &gt; Check &gt; Approve &gt; Accepted</t>
+          <t>슬라이드 46 — Constant List·Metric System은 기능정의서 v0.3 보강 필요</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>M-4-2</t>
+          <t>M-4-1</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
@@ -2096,27 +2096,27 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Work Process</t>
+          <t>Design (DWG)</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>All Department</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-06</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>S-4-1-2</t>
+          <t>S-4-1-1</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>DWG-021, ERP-025</t>
+          <t>DWG-001~016/022~027</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
@@ -2126,12 +2126,12 @@
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K28" s="7" t="inlineStr">
         <is>
-          <t>하위 실체: Design·Manufacturing·Material·Quality (제품별 Work Process Tree)</t>
+          <t>Drawing Editor — 표시 경로: Drawing Info. &gt; Production Design Management &gt; Design &gt; Check &gt; Approve &gt; Accepted</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>M-4-3</t>
+          <t>M-4-2</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
@@ -2151,12 +2151,12 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Design (DWG)</t>
+          <t>Work Process</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>건축 설비 Design</t>
+          <t>All Department</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -2166,27 +2166,27 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>E-4-2</t>
+          <t>S-4-1-2</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>DUCT-001~007</t>
+          <t>DWG-021, ERP-025</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>SETUP·GENERAL</t>
+          <t>SETUP</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
         <is>
-          <t>슬라이드 68 — 사업 범위 확정 대상</t>
+          <t>하위 실체: Design·Manufacturing·Material·Quality (제품별 Work Process Tree)</t>
         </is>
       </c>
     </row>
@@ -2196,52 +2196,52 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>M-5-1</t>
-        </is>
-      </c>
-      <c r="C30" s="12" t="inlineStr">
-        <is>
-          <t>CPQ</t>
+          <t>M-4-3</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>PLM Set-up</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Selection</t>
+          <t>Design (DWG)</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>건축 설비 Design</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>W-02</t>
+          <t>W-15</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>C-1</t>
+          <t>E-4-2</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>CPQ-001~004/007~010</t>
+          <t>DUCT-001~007</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>GENERAL</t>
+          <t>SETUP·GENERAL</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="K30" s="7" t="inlineStr">
         <is>
-          <t>제품 선정</t>
+          <t>슬라이드 68 — 사업 범위 확정 대상</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>M-5-2</t>
+          <t>M-5-1</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
@@ -2261,27 +2261,27 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Technical</t>
+          <t>Selection</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>Product·Item</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>W-03</t>
+          <t>W-02</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>C-2</t>
+          <t>C-1</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>CPQ-005</t>
+          <t>CPQ-001~004/007~010</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
@@ -2291,10 +2291,14 @@
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="K31" s="7" t="inlineStr"/>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K31" s="7" t="inlineStr">
+        <is>
+          <t>제품 선정</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n">
@@ -2302,7 +2306,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>M-5-3</t>
+          <t>M-5-2</t>
         </is>
       </c>
       <c r="C32" s="12" t="inlineStr">
@@ -2312,7 +2316,7 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Document</t>
+          <t>Technical</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
@@ -2322,17 +2326,17 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-03</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>C-3</t>
+          <t>C-2</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>CPQ-006</t>
+          <t>CPQ-005</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
@@ -2353,7 +2357,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>M-5-4</t>
+          <t>M-5-3</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
@@ -2363,12 +2367,12 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Document Management</t>
+          <t>Document</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>문서함 (Set-up→Check→Approve→Accepted)</t>
+          <t>Product·Item</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
@@ -2378,12 +2382,12 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>C-3</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>DOC-001~004</t>
+          <t>CPQ-006</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
@@ -2396,11 +2400,7 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="K33" s="7" t="inlineStr">
-        <is>
-          <t>슬라이드 20/58 breadcrumb — Released Status·Grade 관리</t>
-        </is>
-      </c>
+      <c r="K33" s="7" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n">
@@ -2408,52 +2408,52 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>M-6-1</t>
-        </is>
-      </c>
-      <c r="C34" s="13" t="inlineStr">
-        <is>
-          <t>ERP</t>
+          <t>M-5-4</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>CPQ</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Document Management</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>고객 관리</t>
+          <t>문서함 (Set-up→Check→Approve→Accepted)</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-11</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>§11</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>ERP-015</t>
+          <t>DOC-001~004</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>영업</t>
+          <t>GENERAL</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="K34" s="7" t="inlineStr">
         <is>
-          <t>ERP Toolbar 사용자 편집 가능 (슬라이드 59)</t>
+          <t>슬라이드 20/58 breadcrumb — Released Status·Grade 관리</t>
         </is>
       </c>
     </row>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>M-6-2</t>
+          <t>M-6-1</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
@@ -2478,12 +2478,12 @@
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>Project 등록 (PS)</t>
+          <t>고객 관리</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>W-09</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>ERP-001</t>
+          <t>ERP-015</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">
@@ -2503,10 +2503,14 @@
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="K35" s="7" t="inlineStr"/>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="K35" s="7" t="inlineStr">
+        <is>
+          <t>ERP Toolbar 사용자 편집 가능 (슬라이드 59)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n">
@@ -2514,7 +2518,7 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>M-6-3</t>
+          <t>M-6-2</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
@@ -2529,7 +2533,7 @@
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>Project 관리</t>
+          <t>Project 등록 (PS)</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
@@ -2544,7 +2548,7 @@
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>ERP-001/002</t>
+          <t>ERP-001</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
@@ -2565,7 +2569,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>M-6-4</t>
+          <t>M-6-3</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
@@ -2580,12 +2584,12 @@
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>견적 검토 (PCR)</t>
+          <t>Project 관리</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-09</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
@@ -2595,7 +2599,7 @@
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>CST-005, ERP-004</t>
+          <t>ERP-001/002</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
@@ -2605,7 +2609,7 @@
       </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K37" s="7" t="inlineStr"/>
@@ -2616,7 +2620,7 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>M-6-5</t>
+          <t>M-6-4</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
@@ -2631,7 +2635,7 @@
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>견적 (QCR)</t>
+          <t>견적 검토 (PCR)</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
@@ -2646,7 +2650,7 @@
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>CST-006, ERP-004</t>
+          <t>CST-005, ERP-004</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr">
@@ -2667,7 +2671,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>M-6-6</t>
+          <t>M-6-5</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
@@ -2682,7 +2686,7 @@
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>수주 (OR)</t>
+          <t>견적 (QCR)</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
@@ -2697,7 +2701,7 @@
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>ERP-004</t>
+          <t>CST-006, ERP-004</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
@@ -2707,7 +2711,7 @@
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="K39" s="7" t="inlineStr"/>
@@ -2718,7 +2722,7 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>M-6-7</t>
+          <t>M-6-6</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -2733,7 +2737,7 @@
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>승인 도서 (AP)·고객 승인 (APP)</t>
+          <t>수주 (OR)</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
@@ -2748,7 +2752,7 @@
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>ERP-005</t>
+          <t>ERP-004</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr">
@@ -2769,7 +2773,7 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>M-6-8</t>
+          <t>M-6-7</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -2784,7 +2788,7 @@
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>출고 요청 (FDR)·고객 출고 (SFO)·납품 (DF)</t>
+          <t>승인 도서 (AP)·고객 승인 (APP)</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
@@ -2799,7 +2803,7 @@
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>ERP-009</t>
+          <t>ERP-005</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr">
@@ -2820,7 +2824,7 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>M-6-9</t>
+          <t>M-6-8</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
@@ -2835,7 +2839,7 @@
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>기성 청구 (IR)</t>
+          <t>출고 요청 (FDR)·고객 출고 (SFO)·납품 (DF)</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
@@ -2871,7 +2875,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>M-6-10</t>
+          <t>M-6-9</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
@@ -2886,7 +2890,7 @@
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>시운전 요청 (CR)</t>
+          <t>기성 청구 (IR)</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
@@ -2901,7 +2905,7 @@
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>ERP-010</t>
+          <t>ERP-009</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
@@ -2922,7 +2926,7 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>M-7-1</t>
+          <t>M-6-10</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
@@ -2932,12 +2936,12 @@
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Tech.</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>제작 의뢰 (MR)·제작 점검 (MRR)</t>
+          <t>시운전 요청 (CR)</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
@@ -2952,12 +2956,12 @@
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>ERP-006</t>
+          <t>ERP-010</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>기술</t>
+          <t>영업</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
@@ -2973,7 +2977,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>M-7-2</t>
+          <t>M-7-1</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
@@ -2988,7 +2992,7 @@
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>Part List (PL)·BOM 조회</t>
+          <t>제작 의뢰 (MR)·제작 점검 (MRR)</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
@@ -3003,7 +3007,7 @@
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>RUN-002/010</t>
+          <t>ERP-006</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
@@ -3013,7 +3017,7 @@
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="K45" s="7" t="inlineStr"/>
@@ -3024,7 +3028,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>M-7-3</t>
+          <t>M-7-2</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
@@ -3039,7 +3043,7 @@
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>제품 Set-up (PSU)·자동 제작 설계 (PLM)</t>
+          <t>Part List (PL)·BOM 조회</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
@@ -3054,7 +3058,7 @@
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>RUN-003~005</t>
+          <t>RUN-002/010</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
@@ -3075,7 +3079,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>M-8-1</t>
+          <t>M-7-3</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -3085,12 +3089,12 @@
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Purchasing</t>
+          <t>Tech.</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>구매 관리</t>
+          <t>제품 Set-up (PSU)·자동 제작 설계 (PLM)</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
@@ -3105,17 +3109,17 @@
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>ERP-017/018</t>
+          <t>RUN-003~005</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>자재</t>
+          <t>기술</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K47" s="7" t="inlineStr"/>
@@ -3126,7 +3130,7 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>M-8-2</t>
+          <t>M-8-1</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
@@ -3141,7 +3145,7 @@
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>자재발주요청 (PR)·발주 (PO)</t>
+          <t>구매 관리</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
@@ -3156,7 +3160,7 @@
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>ERP-007</t>
+          <t>ERP-017/018</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
@@ -3177,7 +3181,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>M-8-3</t>
+          <t>M-8-2</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
@@ -3187,12 +3191,12 @@
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Material</t>
+          <t>Purchasing</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>자재 입고 (MI)·출고 (MO)·수령 (RM)</t>
+          <t>자재발주요청 (PR)·발주 (PO)</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
@@ -3228,7 +3232,7 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>M-8-4</t>
+          <t>M-8-3</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
@@ -3243,7 +3247,7 @@
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>재고·창고 관리</t>
+          <t>자재 입고 (MI)·출고 (MO)·수령 (RM)</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
@@ -3258,7 +3262,7 @@
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>ERP-019~021</t>
+          <t>ERP-007</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr">
@@ -3279,7 +3283,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>M-8-5</t>
+          <t>M-8-4</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
@@ -3294,7 +3298,7 @@
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>MRP 자재 소요 계획</t>
+          <t>재고·창고 관리</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
@@ -3309,7 +3313,7 @@
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>ERP-022</t>
+          <t>ERP-019~021</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr">
@@ -3330,7 +3334,7 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>M-8-6</t>
+          <t>M-8-5</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
@@ -3340,12 +3344,12 @@
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Purchasing</t>
+          <t>Material</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>일반 발주 (PR)·구매 승인 (RA)</t>
+          <t>MRP 자재 소요 계획</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
@@ -3360,7 +3364,7 @@
       </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
-          <t>ERP-017</t>
+          <t>ERP-022</t>
         </is>
       </c>
       <c r="I52" s="5" t="inlineStr">
@@ -3373,11 +3377,7 @@
           <t>P5</t>
         </is>
       </c>
-      <c r="K52" s="7" t="inlineStr">
-        <is>
-          <t>슬라이드 10 — 비프로젝트(재작업·공구 등) 구매</t>
-        </is>
-      </c>
+      <c r="K52" s="7" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n">
@@ -3385,7 +3385,7 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>M-9-1</t>
+          <t>M-8-6</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
@@ -3395,12 +3395,12 @@
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Product(생산)</t>
+          <t>Purchasing</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>생산계획 (MP)·Scheduling</t>
+          <t>일반 발주 (PR)·구매 승인 (RA)</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
@@ -3415,12 +3415,12 @@
       </c>
       <c r="H53" s="7" t="inlineStr">
         <is>
-          <t>ERP-023</t>
+          <t>ERP-017</t>
         </is>
       </c>
       <c r="I53" s="5" t="inlineStr">
         <is>
-          <t>생산</t>
+          <t>자재</t>
         </is>
       </c>
       <c r="J53" s="5" t="inlineStr">
@@ -3428,7 +3428,11 @@
           <t>P5</t>
         </is>
       </c>
-      <c r="K53" s="7" t="inlineStr"/>
+      <c r="K53" s="7" t="inlineStr">
+        <is>
+          <t>슬라이드 10 — 비프로젝트(재작업·공구 등) 구매</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n">
@@ -3436,7 +3440,7 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>M-9-2</t>
+          <t>M-9-1</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
@@ -3451,7 +3455,7 @@
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>작업 지시 (WR)</t>
+          <t>생산계획 (MP)·Scheduling</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
@@ -3466,7 +3470,7 @@
       </c>
       <c r="H54" s="7" t="inlineStr">
         <is>
-          <t>ERP-024</t>
+          <t>ERP-023</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
@@ -3487,7 +3491,7 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>M-9-3</t>
+          <t>M-9-2</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
@@ -3502,7 +3506,7 @@
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>공정 관리</t>
+          <t>작업 지시 (WR)</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
@@ -3517,7 +3521,7 @@
       </c>
       <c r="H55" s="7" t="inlineStr">
         <is>
-          <t>ERP-025</t>
+          <t>ERP-024</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
@@ -3538,7 +3542,7 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>M-9-4</t>
+          <t>M-9-3</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
@@ -3553,7 +3557,7 @@
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>반·완성품 (SFI·EF·FF)·Stock 생산 (SPP)</t>
+          <t>공정 관리</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
@@ -3568,7 +3572,7 @@
       </c>
       <c r="H56" s="7" t="inlineStr">
         <is>
-          <t>ERP-008</t>
+          <t>ERP-025</t>
         </is>
       </c>
       <c r="I56" s="5" t="inlineStr">
@@ -3589,7 +3593,7 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>M-9-5</t>
+          <t>M-9-4</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
@@ -3604,7 +3608,7 @@
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>외주 제조 관리</t>
+          <t>반·완성품 (SFI·EF·FF)·Stock 생산 (SPP)</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
@@ -3619,7 +3623,7 @@
       </c>
       <c r="H57" s="7" t="inlineStr">
         <is>
-          <t>ERP-030</t>
+          <t>ERP-008</t>
         </is>
       </c>
       <c r="I57" s="5" t="inlineStr">
@@ -3640,7 +3644,7 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>M-9-6</t>
+          <t>M-9-5</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
@@ -3655,7 +3659,7 @@
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>재작업 요청 (WR)</t>
+          <t>외주 제조 관리</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
@@ -3670,7 +3674,7 @@
       </c>
       <c r="H58" s="7" t="inlineStr">
         <is>
-          <t>ERP-029/030</t>
+          <t>ERP-030</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
@@ -3683,11 +3687,7 @@
           <t>P5</t>
         </is>
       </c>
-      <c r="K58" s="7" t="inlineStr">
-        <is>
-          <t>슬라이드 10</t>
-        </is>
-      </c>
+      <c r="K58" s="7" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n">
@@ -3695,7 +3695,7 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>M-10-1</t>
+          <t>M-9-6</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
@@ -3705,12 +3705,12 @@
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>Product(생산)</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>자재 품질 검사 (ER)</t>
+          <t>재작업 요청 (WR)</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
@@ -3725,12 +3725,12 @@
       </c>
       <c r="H59" s="7" t="inlineStr">
         <is>
-          <t>ERP-027</t>
+          <t>ERP-029/030</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>생산</t>
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr">
@@ -3738,7 +3738,11 @@
           <t>P5</t>
         </is>
       </c>
-      <c r="K59" s="7" t="inlineStr"/>
+      <c r="K59" s="7" t="inlineStr">
+        <is>
+          <t>슬라이드 10</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n">
@@ -3746,7 +3750,7 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>M-10-2</t>
+          <t>M-10-1</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
@@ -3761,7 +3765,7 @@
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>반·완성품 검사 (EF)</t>
+          <t>자재 품질 검사 (ER)</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
@@ -3797,7 +3801,7 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>M-10-3</t>
+          <t>M-10-2</t>
         </is>
       </c>
       <c r="C61" s="13" t="inlineStr">
@@ -3812,7 +3816,7 @@
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>부적합 처리 (NCF)</t>
+          <t>반·완성품 검사 (EF)</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
@@ -3827,7 +3831,7 @@
       </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
-          <t>ERP-012</t>
+          <t>ERP-027</t>
         </is>
       </c>
       <c r="I61" s="5" t="inlineStr">
@@ -3848,7 +3852,7 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>M-10-4</t>
+          <t>M-10-3</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
@@ -3863,7 +3867,7 @@
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>인증서 발급 (CR)</t>
+          <t>부적합 처리 (NCF)</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
@@ -3878,7 +3882,7 @@
       </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
-          <t>ERP-030</t>
+          <t>ERP-012</t>
         </is>
       </c>
       <c r="I62" s="5" t="inlineStr">
@@ -3891,11 +3895,7 @@
           <t>P5</t>
         </is>
       </c>
-      <c r="K62" s="7" t="inlineStr">
-        <is>
-          <t>슬라이드 10</t>
-        </is>
-      </c>
+      <c r="K62" s="7" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>M-11-1</t>
+          <t>M-10-4</t>
         </is>
       </c>
       <c r="C63" s="13" t="inlineStr">
@@ -3913,12 +3913,12 @@
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>A/S</t>
+          <t>QC</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>시운전 (CF)</t>
+          <t>인증서 발급 (CR)</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
@@ -3933,12 +3933,12 @@
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>ERP-010</t>
+          <t>ERP-030</t>
         </is>
       </c>
       <c r="I63" s="5" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>QC</t>
         </is>
       </c>
       <c r="J63" s="5" t="inlineStr">
@@ -3946,7 +3946,11 @@
           <t>P5</t>
         </is>
       </c>
-      <c r="K63" s="7" t="inlineStr"/>
+      <c r="K63" s="7" t="inlineStr">
+        <is>
+          <t>슬라이드 10</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n">
@@ -3954,7 +3958,7 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>M-11-2</t>
+          <t>M-11-1</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
@@ -3969,7 +3973,7 @@
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>유지보수</t>
+          <t>시운전 (CF)</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
@@ -3984,7 +3988,7 @@
       </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>APP-006</t>
+          <t>ERP-010</t>
         </is>
       </c>
       <c r="I64" s="5" t="inlineStr">
@@ -4005,7 +4009,7 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>M-12-1</t>
+          <t>M-11-2</t>
         </is>
       </c>
       <c r="C65" s="13" t="inlineStr">
@@ -4015,12 +4019,12 @@
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>A/S</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>세금계산 매입 (II)·매출 (IO)</t>
+          <t>유지보수</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
@@ -4035,12 +4039,12 @@
       </c>
       <c r="H65" s="7" t="inlineStr">
         <is>
-          <t>ERP-011</t>
+          <t>APP-006</t>
         </is>
       </c>
       <c r="I65" s="5" t="inlineStr">
         <is>
-          <t>재무</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="J65" s="5" t="inlineStr">
@@ -4056,7 +4060,7 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>M-12-2</t>
+          <t>M-12-1</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
@@ -4071,7 +4075,7 @@
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>매입 출금 (PA)·매출 입금 (PI)</t>
+          <t>세금계산 매입 (II)·매출 (IO)</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr">
@@ -4107,7 +4111,7 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>M-12-3</t>
+          <t>M-12-2</t>
         </is>
       </c>
       <c r="C67" s="13" t="inlineStr">
@@ -4122,7 +4126,7 @@
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>정산 (RR)·정산승인 (RA)·재무관리 (FM)</t>
+          <t>매입 출금 (PA)·매출 입금 (PI)</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
@@ -4158,7 +4162,7 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>M-12-4</t>
+          <t>M-12-3</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
@@ -4173,7 +4177,7 @@
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>Advance 선지급 (AR)</t>
+          <t>정산 (RR)·정산승인 (RA)·재무관리 (FM)</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr">
@@ -4201,11 +4205,7 @@
           <t>P5</t>
         </is>
       </c>
-      <c r="K68" s="7" t="inlineStr">
-        <is>
-          <t>슬라이드 10 — 기능정의서 v0.3 보강 필요</t>
-        </is>
-      </c>
+      <c r="K68" s="7" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="5" t="n">
@@ -4213,7 +4213,7 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>M-13-1</t>
+          <t>M-12-4</t>
         </is>
       </c>
       <c r="C69" s="13" t="inlineStr">
@@ -4223,12 +4223,12 @@
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>임직원 관리·임직원 출금 (CO)</t>
+          <t>Advance 선지급 (AR)</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
@@ -4243,12 +4243,12 @@
       </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ERP-011</t>
         </is>
       </c>
       <c r="I69" s="5" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>재무</t>
         </is>
       </c>
       <c r="J69" s="5" t="inlineStr">
@@ -4258,7 +4258,7 @@
       </c>
       <c r="K69" s="7" t="inlineStr">
         <is>
-          <t>상세 v0.3</t>
+          <t>슬라이드 10 — 기능정의서 v0.3 보강 필요</t>
         </is>
       </c>
     </row>
@@ -4268,7 +4268,7 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>M-14-1</t>
+          <t>M-12-5</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
@@ -4278,40 +4278,44 @@
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>Company Info.</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>ERP System·Department</t>
+          <t>단가 관리 (견적·구매이력·재고단가·견적적용)</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-13</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>§11</t>
+          <t>D-3/D-4</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr">
         <is>
-          <t>SYS-019/020</t>
+          <t>CST-001, ERP-021</t>
         </is>
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>재무·자재</t>
         </is>
       </c>
       <c r="J70" s="5" t="inlineStr">
         <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="K70" s="7" t="inlineStr"/>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="K70" s="7" t="inlineStr">
+        <is>
+          <t>슬라이드 74/75 단가 관리 Table</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="n">
@@ -4319,7 +4323,7 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>M-14-2</t>
+          <t>M-13-1</t>
         </is>
       </c>
       <c r="C71" s="13" t="inlineStr">
@@ -4329,12 +4333,12 @@
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>Company Info.</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>Company DB (고객·공급·파트너·은행)</t>
+          <t>임직원 관리·임직원 출금 (CO)</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
@@ -4349,20 +4353,24 @@
       </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
-          <t>ERP-015</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I71" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="J71" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="K71" s="7" t="inlineStr"/>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="K71" s="7" t="inlineStr">
+        <is>
+          <t>상세 v0.3</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="n">
@@ -4370,7 +4378,7 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>M-14-3</t>
+          <t>M-14-1</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
@@ -4385,7 +4393,7 @@
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>업체 평가 (CE)·Project 평가 (PE)</t>
+          <t>ERP System·Department</t>
         </is>
       </c>
       <c r="F72" s="5" t="inlineStr">
@@ -4400,7 +4408,7 @@
       </c>
       <c r="H72" s="7" t="inlineStr">
         <is>
-          <t>ERP-013</t>
+          <t>SYS-019/020</t>
         </is>
       </c>
       <c r="I72" s="5" t="inlineStr">
@@ -4421,7 +4429,7 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>M-14-4</t>
+          <t>M-14-2</t>
         </is>
       </c>
       <c r="C73" s="13" t="inlineStr">
@@ -4436,12 +4444,12 @@
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Company DB (고객·공급·파트너·은행)</t>
         </is>
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>W-10</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
@@ -4451,17 +4459,17 @@
       </c>
       <c r="H73" s="7" t="inlineStr">
         <is>
-          <t>ERP-014</t>
+          <t>ERP-015</t>
         </is>
       </c>
       <c r="I73" s="5" t="inlineStr">
         <is>
-          <t>ADMIN·경영</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="J73" s="5" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K73" s="7" t="inlineStr"/>
@@ -4472,7 +4480,7 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>M-14-5</t>
+          <t>M-14-3</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
@@ -4487,7 +4495,7 @@
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>PCR 기준 관리</t>
+          <t>업체 평가 (CE)·Project 평가 (PE)</t>
         </is>
       </c>
       <c r="F74" s="5" t="inlineStr">
@@ -4502,24 +4510,20 @@
       </c>
       <c r="H74" s="7" t="inlineStr">
         <is>
-          <t>CST-005</t>
+          <t>ERP-013</t>
         </is>
       </c>
       <c r="I74" s="5" t="inlineStr">
         <is>
-          <t>ADMIN·재무</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="J74" s="5" t="inlineStr">
         <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="K74" s="7" t="inlineStr">
-        <is>
-          <t>슬라이드 18 — Company info. 하위 3. PCR</t>
-        </is>
-      </c>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="K74" s="7" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="5" t="n">
@@ -4527,7 +4531,7 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>M-14-6</t>
+          <t>M-14-4</t>
         </is>
       </c>
       <c r="C75" s="13" t="inlineStr">
@@ -4542,39 +4546,35 @@
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>Access Control·Version Management</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-10</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>D-1</t>
+          <t>§11</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr">
         <is>
-          <t>SYS-003~005/012</t>
+          <t>ERP-014</t>
         </is>
       </c>
       <c r="I75" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>ADMIN·경영</t>
         </is>
       </c>
       <c r="J75" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="K75" s="7" t="inlineStr">
-        <is>
-          <t>슬라이드 72 — 권한 설정·버전 관리</t>
-        </is>
-      </c>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="K75" s="7" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="5" t="n">
@@ -4582,52 +4582,52 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>M-15-1</t>
-        </is>
-      </c>
-      <c r="C76" s="14" t="inlineStr">
-        <is>
-          <t>공통</t>
+          <t>M-14-5</t>
+        </is>
+      </c>
+      <c r="C76" s="13" t="inlineStr">
+        <is>
+          <t>ERP</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>로그인</t>
+          <t>Company Info.</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>PCR 기준 관리</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>W-01</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>§11</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr">
         <is>
-          <t>SYS-001/002</t>
+          <t>CST-005</t>
         </is>
       </c>
       <c r="I76" s="5" t="inlineStr">
         <is>
-          <t>전체</t>
+          <t>ADMIN·재무</t>
         </is>
       </c>
       <c r="J76" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="K76" s="7" t="inlineStr">
         <is>
-          <t>슬라이드 3</t>
+          <t>슬라이드 18 — Company info. 하위 3. PCR</t>
         </is>
       </c>
     </row>
@@ -4637,22 +4637,22 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>M-15-2</t>
-        </is>
-      </c>
-      <c r="C77" s="14" t="inlineStr">
-        <is>
-          <t>공통</t>
+          <t>M-14-6</t>
+        </is>
+      </c>
+      <c r="C77" s="13" t="inlineStr">
+        <is>
+          <t>ERP</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>승인함</t>
+          <t>Company Info.</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>승인 요청·처리·이력</t>
+          <t>Access Control·Version Management</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
@@ -4662,17 +4662,17 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>D-1</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
-          <t>SYS-009~011</t>
+          <t>SYS-003~005/012</t>
         </is>
       </c>
       <c r="I77" s="5" t="inlineStr">
         <is>
-          <t>전체</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="J77" s="5" t="inlineStr">
@@ -4682,7 +4682,7 @@
       </c>
       <c r="K77" s="7" t="inlineStr">
         <is>
-          <t>좌측 하단 위젯 + 전용 화면</t>
+          <t>슬라이드 72 — 권한 설정·버전 관리</t>
         </is>
       </c>
     </row>
@@ -4692,50 +4692,54 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>M-15-3</t>
-        </is>
-      </c>
-      <c r="C78" s="14" t="inlineStr">
-        <is>
-          <t>공통</t>
+          <t>M-14-7</t>
+        </is>
+      </c>
+      <c r="C78" s="13" t="inlineStr">
+        <is>
+          <t>ERP</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>일정·To-do</t>
+          <t>Company Info.</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>Schedule·To-do·Done</t>
+          <t>ERP Process Set-up</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-14</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
-          <t>E-3</t>
+          <t>슬라이드17 5-1</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr">
         <is>
-          <t>SYS-017</t>
+          <t>ERP-002, SVC-09</t>
         </is>
       </c>
       <c r="I78" s="5" t="inlineStr">
         <is>
-          <t>전체</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="J78" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="K78" s="7" t="inlineStr"/>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="K78" s="7" t="inlineStr">
+        <is>
+          <t>프로세스 정의(선행·후행·자동) 관리</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="n">
@@ -4743,22 +4747,22 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>M-15-4</t>
-        </is>
-      </c>
-      <c r="C79" s="14" t="inlineStr">
-        <is>
-          <t>공통</t>
+          <t>M-14-8</t>
+        </is>
+      </c>
+      <c r="C79" s="13" t="inlineStr">
+        <is>
+          <t>ERP</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>알림</t>
+          <t>Company Info.</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>알림 목록·공지</t>
+          <t>ERP DB Set-up</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
@@ -4768,25 +4772,29 @@
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>슬라이드17 5-2</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
-          <t>SYS-013/014</t>
+          <t>SYS-019/020</t>
         </is>
       </c>
       <c r="I79" s="5" t="inlineStr">
         <is>
-          <t>전체</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="J79" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="K79" s="7" t="inlineStr"/>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="K79" s="7" t="inlineStr">
+        <is>
+          <t>기능정의서 v0.3 보강 필요</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="n">
@@ -4794,22 +4802,22 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>M-15-5</t>
-        </is>
-      </c>
-      <c r="C80" s="14" t="inlineStr">
-        <is>
-          <t>공통</t>
+          <t>M-14-9</t>
+        </is>
+      </c>
+      <c r="C80" s="13" t="inlineStr">
+        <is>
+          <t>ERP</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>업무 소통</t>
+          <t>Company Info.</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>Project 중심 대화 (SNS)</t>
+          <t>ERP Form Set-up (EDIM Toolbox)</t>
         </is>
       </c>
       <c r="F80" s="5" t="inlineStr">
@@ -4819,17 +4827,17 @@
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>슬라이드17 5-3</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr">
         <is>
-          <t>SYS-018</t>
+          <t>ERP-016, TBX-003</t>
         </is>
       </c>
       <c r="I80" s="5" t="inlineStr">
         <is>
-          <t>전체</t>
+          <t>ADMIN·SETUP</t>
         </is>
       </c>
       <c r="J80" s="5" t="inlineStr">
@@ -4837,11 +4845,7 @@
           <t>P5</t>
         </is>
       </c>
-      <c r="K80" s="7" t="inlineStr">
-        <is>
-          <t>슬라이드 57</t>
-        </is>
-      </c>
+      <c r="K80" s="7" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="n">
@@ -4849,22 +4853,22 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>M-15-6</t>
-        </is>
-      </c>
-      <c r="C81" s="14" t="inlineStr">
-        <is>
-          <t>공통</t>
+          <t>M-14-10</t>
+        </is>
+      </c>
+      <c r="C81" s="13" t="inlineStr">
+        <is>
+          <t>ERP</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>검색</t>
+          <t>Company Info.</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>Hierarchy·자료 통합 검색</t>
+          <t>보안 설정 (Security Solution)</t>
         </is>
       </c>
       <c r="F81" s="5" t="inlineStr">
@@ -4874,25 +4878,29 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>E-3</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr">
         <is>
-          <t>SYS-006</t>
+          <t>DOC-004</t>
         </is>
       </c>
       <c r="I81" s="5" t="inlineStr">
         <is>
-          <t>전체</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="J81" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="K81" s="7" t="inlineStr"/>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="K81" s="7" t="inlineStr">
+        <is>
+          <t>슬라이드 58 placeholder — 요건 고객 협의</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="n">
@@ -4900,7 +4908,7 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>M-15-7</t>
+          <t>M-15-1</t>
         </is>
       </c>
       <c r="C82" s="14" t="inlineStr">
@@ -4910,27 +4918,27 @@
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>개인 설정</t>
+          <t>로그인</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>색상·언어·판넬 화면 조정</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-01</t>
         </is>
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>E-1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr">
         <is>
-          <t>SYS-016</t>
+          <t>SYS-001/002</t>
         </is>
       </c>
       <c r="I82" s="5" t="inlineStr">
@@ -4940,12 +4948,12 @@
       </c>
       <c r="J82" s="5" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K82" s="7" t="inlineStr">
         <is>
-          <t>슬라이드 57 — Frame/Canvas 색상, 아코디언·펼침</t>
+          <t>슬라이드 3</t>
         </is>
       </c>
     </row>
@@ -4955,7 +4963,7 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>M-15-8</t>
+          <t>M-15-2</t>
         </is>
       </c>
       <c r="C83" s="14" t="inlineStr">
@@ -4965,27 +4973,27 @@
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>Project Folder</t>
+          <t>승인함</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>산출물 탐색 (DWG·Price·Data·BOM)</t>
+          <t>승인 요청·처리·이력</t>
         </is>
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-12</t>
         </is>
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>E-3</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr">
         <is>
-          <t>RUN-009</t>
+          <t>SYS-009~011</t>
         </is>
       </c>
       <c r="I83" s="5" t="inlineStr">
@@ -4995,12 +5003,12 @@
       </c>
       <c r="J83" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K83" s="7" t="inlineStr">
         <is>
-          <t>슬라이드 64 Hierarchy List 4. Project</t>
+          <t>좌측 하단 위젯 + 전용 화면</t>
         </is>
       </c>
     </row>
@@ -5010,22 +5018,22 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>M-16-1</t>
-        </is>
-      </c>
-      <c r="C84" s="15" t="inlineStr">
-        <is>
-          <t>Mobile App</t>
+          <t>M-15-3</t>
+        </is>
+      </c>
+      <c r="C84" s="14" t="inlineStr">
+        <is>
+          <t>공통</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>QR</t>
+          <t>일정·To-do</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>QR 정보 열람 (도면·서류·Project·업무)</t>
+          <t>Schedule·To-do·Done</t>
         </is>
       </c>
       <c r="F84" s="5" t="inlineStr">
@@ -5035,12 +5043,12 @@
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>§12</t>
+          <t>E-3</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr">
         <is>
-          <t>APP-001</t>
+          <t>SYS-017</t>
         </is>
       </c>
       <c r="I84" s="5" t="inlineStr">
@@ -5050,7 +5058,7 @@
       </c>
       <c r="J84" s="5" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K84" s="7" t="inlineStr"/>
@@ -5061,22 +5069,22 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>M-16-2</t>
-        </is>
-      </c>
-      <c r="C85" s="15" t="inlineStr">
-        <is>
-          <t>Mobile App</t>
+          <t>M-15-4</t>
+        </is>
+      </c>
+      <c r="C85" s="14" t="inlineStr">
+        <is>
+          <t>공통</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>알림</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>업무 승인</t>
+          <t>알림 목록·공지</t>
         </is>
       </c>
       <c r="F85" s="5" t="inlineStr">
@@ -5086,22 +5094,22 @@
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>§12</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr">
         <is>
-          <t>APP-002</t>
+          <t>SYS-013/014</t>
         </is>
       </c>
       <c r="I85" s="5" t="inlineStr">
         <is>
-          <t>ADMIN↑</t>
+          <t>전체</t>
         </is>
       </c>
       <c r="J85" s="5" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K85" s="7" t="inlineStr"/>
@@ -5112,22 +5120,22 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>M-16-3</t>
-        </is>
-      </c>
-      <c r="C86" s="15" t="inlineStr">
-        <is>
-          <t>Mobile App</t>
+          <t>M-15-5</t>
+        </is>
+      </c>
+      <c r="C86" s="14" t="inlineStr">
+        <is>
+          <t>공통</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>소통</t>
+          <t>업무 소통</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>Project 중심 대화·History</t>
+          <t>Project 중심 대화 (SNS)</t>
         </is>
       </c>
       <c r="F86" s="5" t="inlineStr">
@@ -5137,12 +5145,12 @@
       </c>
       <c r="G86" s="5" t="inlineStr">
         <is>
-          <t>§12</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H86" s="7" t="inlineStr">
         <is>
-          <t>APP-003</t>
+          <t>SYS-018</t>
         </is>
       </c>
       <c r="I86" s="5" t="inlineStr">
@@ -5155,7 +5163,11 @@
           <t>P5</t>
         </is>
       </c>
-      <c r="K86" s="7" t="inlineStr"/>
+      <c r="K86" s="7" t="inlineStr">
+        <is>
+          <t>슬라이드 57</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="n">
@@ -5163,22 +5175,22 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>M-16-4</t>
-        </is>
-      </c>
-      <c r="C87" s="15" t="inlineStr">
-        <is>
-          <t>Mobile App</t>
+          <t>M-15-6</t>
+        </is>
+      </c>
+      <c r="C87" s="14" t="inlineStr">
+        <is>
+          <t>공통</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>자재</t>
+          <t>검색</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>자재 입출고</t>
+          <t>Hierarchy·자료 통합 검색</t>
         </is>
       </c>
       <c r="F87" s="5" t="inlineStr">
@@ -5188,22 +5200,22 @@
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>§12</t>
+          <t>E-3</t>
         </is>
       </c>
       <c r="H87" s="7" t="inlineStr">
         <is>
-          <t>APP-004</t>
+          <t>SYS-006</t>
         </is>
       </c>
       <c r="I87" s="5" t="inlineStr">
         <is>
-          <t>자재</t>
+          <t>전체</t>
         </is>
       </c>
       <c r="J87" s="5" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K87" s="7" t="inlineStr"/>
@@ -5214,22 +5226,22 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>M-16-5</t>
-        </is>
-      </c>
-      <c r="C88" s="15" t="inlineStr">
-        <is>
-          <t>Mobile App</t>
+          <t>M-15-7</t>
+        </is>
+      </c>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>공통</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>검수</t>
+          <t>개인 설정</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>자재·완성품·설치완료 검수</t>
+          <t>색상·언어·판넬 화면 조정</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr">
@@ -5239,25 +5251,29 @@
       </c>
       <c r="G88" s="5" t="inlineStr">
         <is>
-          <t>§12</t>
+          <t>E-1</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr">
         <is>
-          <t>APP-005</t>
+          <t>SYS-016</t>
         </is>
       </c>
       <c r="I88" s="5" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>전체</t>
         </is>
       </c>
       <c r="J88" s="5" t="inlineStr">
         <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="K88" s="7" t="inlineStr"/>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="K88" s="7" t="inlineStr">
+        <is>
+          <t>슬라이드 57 — Frame/Canvas 색상, 아코디언·펼침</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="n">
@@ -5265,22 +5281,22 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>M-16-6</t>
-        </is>
-      </c>
-      <c r="C89" s="15" t="inlineStr">
-        <is>
-          <t>Mobile App</t>
+          <t>M-15-8</t>
+        </is>
+      </c>
+      <c r="C89" s="14" t="inlineStr">
+        <is>
+          <t>공통</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>유지보수</t>
+          <t>Project Folder</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>Client 유지보수 접수·처리</t>
+          <t>산출물 탐색 (DWG·Price·Data·BOM)</t>
         </is>
       </c>
       <c r="F89" s="5" t="inlineStr">
@@ -5290,25 +5306,29 @@
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>§12</t>
+          <t>E-3</t>
         </is>
       </c>
       <c r="H89" s="7" t="inlineStr">
         <is>
-          <t>APP-006</t>
+          <t>RUN-009</t>
         </is>
       </c>
       <c r="I89" s="5" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>전체</t>
         </is>
       </c>
       <c r="J89" s="5" t="inlineStr">
         <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="K89" s="7" t="inlineStr"/>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K89" s="7" t="inlineStr">
+        <is>
+          <t>슬라이드 64 Hierarchy List 4. Project</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="n">
@@ -5316,22 +5336,22 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>M-16-7</t>
-        </is>
-      </c>
-      <c r="C90" s="15" t="inlineStr">
-        <is>
-          <t>Mobile App</t>
+          <t>M-15-9</t>
+        </is>
+      </c>
+      <c r="C90" s="14" t="inlineStr">
+        <is>
+          <t>공통</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>이력 조회</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>공지·알림 수신</t>
+          <t>생성·편집·삭제·승인 History</t>
         </is>
       </c>
       <c r="F90" s="5" t="inlineStr">
@@ -5341,25 +5361,29 @@
       </c>
       <c r="G90" s="5" t="inlineStr">
         <is>
-          <t>§12</t>
+          <t>D-1</t>
         </is>
       </c>
       <c r="H90" s="7" t="inlineStr">
         <is>
-          <t>APP-007</t>
+          <t>SYS-012</t>
         </is>
       </c>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>전체</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="J90" s="5" t="inlineStr">
         <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="K90" s="7" t="inlineStr"/>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K90" s="7" t="inlineStr">
+        <is>
+          <t>슬라이드 57 History 관리·슬라이드 72 Version management</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="n">
@@ -5367,57 +5391,414 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
+          <t>M-16-1</t>
+        </is>
+      </c>
+      <c r="C91" s="15" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="D91" s="7" t="inlineStr">
+        <is>
+          <t>QR</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="inlineStr">
+        <is>
+          <t>QR 정보 열람 (도면·서류·Project·업무)</t>
+        </is>
+      </c>
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>W-16</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>§12</t>
+        </is>
+      </c>
+      <c r="H91" s="7" t="inlineStr">
+        <is>
+          <t>APP-001</t>
+        </is>
+      </c>
+      <c r="I91" s="5" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="J91" s="5" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="K91" s="7" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>M-16-2</t>
+        </is>
+      </c>
+      <c r="C92" s="15" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="inlineStr">
+        <is>
+          <t>승인</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>업무 승인</t>
+        </is>
+      </c>
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>W-16</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>§12</t>
+        </is>
+      </c>
+      <c r="H92" s="7" t="inlineStr">
+        <is>
+          <t>APP-002</t>
+        </is>
+      </c>
+      <c r="I92" s="5" t="inlineStr">
+        <is>
+          <t>ADMIN↑</t>
+        </is>
+      </c>
+      <c r="J92" s="5" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="K92" s="7" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>M-16-3</t>
+        </is>
+      </c>
+      <c r="C93" s="15" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="D93" s="7" t="inlineStr">
+        <is>
+          <t>소통</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="inlineStr">
+        <is>
+          <t>Project 중심 대화·History</t>
+        </is>
+      </c>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>§12</t>
+        </is>
+      </c>
+      <c r="H93" s="7" t="inlineStr">
+        <is>
+          <t>APP-003</t>
+        </is>
+      </c>
+      <c r="I93" s="5" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="J93" s="5" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="K93" s="7" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>M-16-4</t>
+        </is>
+      </c>
+      <c r="C94" s="15" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="D94" s="7" t="inlineStr">
+        <is>
+          <t>자재</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="inlineStr">
+        <is>
+          <t>자재 입출고</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>§12</t>
+        </is>
+      </c>
+      <c r="H94" s="7" t="inlineStr">
+        <is>
+          <t>APP-004</t>
+        </is>
+      </c>
+      <c r="I94" s="5" t="inlineStr">
+        <is>
+          <t>자재</t>
+        </is>
+      </c>
+      <c r="J94" s="5" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="K94" s="7" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>M-16-5</t>
+        </is>
+      </c>
+      <c r="C95" s="15" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="D95" s="7" t="inlineStr">
+        <is>
+          <t>검수</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="inlineStr">
+        <is>
+          <t>자재·완성품·설치완료 검수</t>
+        </is>
+      </c>
+      <c r="F95" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>§12</t>
+        </is>
+      </c>
+      <c r="H95" s="7" t="inlineStr">
+        <is>
+          <t>APP-005</t>
+        </is>
+      </c>
+      <c r="I95" s="5" t="inlineStr">
+        <is>
+          <t>QC</t>
+        </is>
+      </c>
+      <c r="J95" s="5" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="K95" s="7" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>M-16-6</t>
+        </is>
+      </c>
+      <c r="C96" s="15" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="D96" s="7" t="inlineStr">
+        <is>
+          <t>유지보수</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="inlineStr">
+        <is>
+          <t>Client 유지보수 접수·처리</t>
+        </is>
+      </c>
+      <c r="F96" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="inlineStr">
+        <is>
+          <t>§12</t>
+        </is>
+      </c>
+      <c r="H96" s="7" t="inlineStr">
+        <is>
+          <t>APP-006</t>
+        </is>
+      </c>
+      <c r="I96" s="5" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J96" s="5" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="K96" s="7" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>M-16-7</t>
+        </is>
+      </c>
+      <c r="C97" s="15" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="D97" s="7" t="inlineStr">
+        <is>
+          <t>공지</t>
+        </is>
+      </c>
+      <c r="E97" s="7" t="inlineStr">
+        <is>
+          <t>공지·알림 수신</t>
+        </is>
+      </c>
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="inlineStr">
+        <is>
+          <t>§12</t>
+        </is>
+      </c>
+      <c r="H97" s="7" t="inlineStr">
+        <is>
+          <t>APP-007</t>
+        </is>
+      </c>
+      <c r="I97" s="5" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="J97" s="5" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="K97" s="7" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
           <t>M-16-8</t>
         </is>
       </c>
-      <c r="C91" s="15" t="inlineStr">
+      <c r="C98" s="15" t="inlineStr">
         <is>
           <t>Mobile App</t>
         </is>
       </c>
-      <c r="D91" s="7" t="inlineStr">
+      <c r="D98" s="7" t="inlineStr">
         <is>
           <t>AR</t>
         </is>
       </c>
-      <c r="E91" s="7" t="inlineStr">
+      <c r="E98" s="7" t="inlineStr">
         <is>
           <t>증강현실 View</t>
         </is>
       </c>
-      <c r="F91" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G91" s="5" t="inlineStr">
+      <c r="F98" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G98" s="5" t="inlineStr">
         <is>
           <t>§12</t>
         </is>
       </c>
-      <c r="H91" s="7" t="inlineStr">
+      <c r="H98" s="7" t="inlineStr">
         <is>
           <t>APP-008</t>
         </is>
       </c>
-      <c r="I91" s="5" t="inlineStr">
+      <c r="I98" s="5" t="inlineStr">
         <is>
           <t>현장</t>
         </is>
       </c>
-      <c r="J91" s="5" t="inlineStr">
+      <c r="J98" s="5" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="K91" s="7" t="inlineStr">
+      <c r="K98" s="7" t="inlineStr">
         <is>
           <t>후순위</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K91"/>
+  <autoFilter ref="A1:K98"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
edim-ai-blueprint: 화면설계서 v0.3 — 누락 화면 8종 추가 (16→24)
- W-17 CPQ Document(C-3, 슬라이드8) · W-18 Print Set-up(S-3-4, 슬라이드50 — 양식 캔버스·워터마크)
- W-19 Work Process 공정(S-4-1-2, 슬라이드44/45 — MAKE/BUY·제조비 입력)
- W-20 데이터 Table 관리(row_key_num 규칙 노출) · W-21 구매·발주(슬라이드53 — 단가 resolve·공급자 코드)
- W-22 부서 업무함(선행검사·기한경고) · W-23 사용자·권한 관리(매트릭스 편집)
- W-24 Project Folder·이력(v0.4 folder 규약·sys_history diff)
- 메뉴정의서 화면 ID 9건 배정 → 권한·RTM 연쇄 재생성 (178/178 유지)
- 신규 화면 렌더 검증 (W-18/W-24 스크린샷)
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_메뉴정의서.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_메뉴정의서.xlsx
@@ -1635,7 +1635,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-18</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-20</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-19</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-17</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-21</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-23</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
@@ -5038,7 +5038,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-22</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
@@ -5301,7 +5301,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-24</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
@@ -5356,7 +5356,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-24</t>
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr">

</xml_diff>